<commit_message>
v434.0.0: Aktenausgabe und Rechtsstand konsolidieren
</commit_message>
<xml_diff>
--- a/testakten/beamtenrecht-richterlaufbahn-besoldung-mondsee/51-besoldungs-und-fristenmodell-erweitert.xlsx
+++ b/testakten/beamtenrecht-richterlaufbahn-besoldung-mondsee/51-besoldungs-und-fristenmodell-erweitert.xlsx
@@ -430,12 +430,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>R1 brutto fiktiv</t>
+          <t>R1 brutto Szenario</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>R2 brutto fiktiv</t>
+          <t>R2 brutto Szenario</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -462,7 +462,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -492,7 +492,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -522,7 +522,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -552,7 +552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -582,7 +582,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -612,7 +612,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -642,7 +642,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -702,7 +702,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -732,7 +732,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -762,7 +762,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -792,7 +792,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>fiktiv bei erfolgreicher Neubescheidung</t>
+          <t>Szenario bei erfolgreicher Neubescheidung</t>
         </is>
       </c>
       <c r="C13" t="n">

</xml_diff>